<commit_message>
Scenario/BAU fixes: H2 production shares, gas price FoPITY inclusion
</commit_message>
<xml_diff>
--- a/InputData/hydgn/BHPSbP/BAU Hydrogen Production Shr by Pathway.xlsx
+++ b/InputData/hydgn/BHPSbP/BAU Hydrogen Production Shr by Pathway.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\hydgn\BHPSbP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0746773-3F94-4C80-9392-DDC2F80141A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C64BE0A-0A22-4081-AE98-1D3A0E06D094}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1520" yWindow="1520" windowWidth="14400" windowHeight="9340" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="38">
   <si>
     <t>BHPSbP BAU Hydrogen Production Shares by Pathway</t>
   </si>
@@ -157,6 +157,24 @@
   </si>
   <si>
     <t>pgs. 10, 16</t>
+  </si>
+  <si>
+    <t>blue share of clean H2 supply</t>
+  </si>
+  <si>
+    <t>Hydrogen Supply Outlook Update: 10% Cut</t>
+  </si>
+  <si>
+    <t>https://www.bnef.com/insights/38875</t>
+  </si>
+  <si>
+    <t>Blue/green clean hydrogen split</t>
+  </si>
+  <si>
+    <t>Clean hydrogen offtake demand</t>
+  </si>
+  <si>
+    <t>Aggregated expected production from projects; included with permission</t>
   </si>
 </sst>
 </file>
@@ -166,7 +184,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -190,8 +208,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -201,6 +226,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -214,11 +245,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -232,10 +264,14 @@
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -261,16 +297,16 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>536696</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>70110</xdr:rowOff>
+      <xdr:colOff>534092</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>171193</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2">
+        <xdr:cNvPr id="4" name="Picture 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D8661492-DC81-408D-BF1C-FD0AB9692D4E}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{150E1DB1-3649-4488-8F2D-F0C181554476}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -286,52 +322,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="609600" y="184150"/>
-          <a:ext cx="6023096" cy="3384810"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>534092</xdr:colOff>
-      <xdr:row>37</xdr:row>
-      <xdr:rowOff>171193</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Picture 4">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{02F6FC29-38EA-45AA-81F7-E95FC535D07A}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="606136" y="3752273"/>
-          <a:ext cx="5989320" cy="3360625"/>
+          <a:off x="606136" y="184006"/>
+          <a:ext cx="5989320" cy="3299289"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -606,10 +598,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.7265625" customWidth="1"/>
+    <col min="2" max="2" width="52.6328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
@@ -621,28 +614,63 @@
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="10" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B4" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B4" s="3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B5" s="3">
         <v>2025</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B5" t="s">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B6" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B6" s="4" t="s">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B7" s="4" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B7" t="s">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B8" t="s">
         <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B10" s="10" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B11" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B12" s="3">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B13" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B14" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B15" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -653,25 +681,25 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3FCF00DD-FBB5-4F2F-A64F-4218B001AAAE}">
-  <dimension ref="L3:O16"/>
+  <dimension ref="B3:AM35"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="3" spans="12:15" x14ac:dyDescent="0.35">
       <c r="M3" t="s">
         <v>10</v>
       </c>
-      <c r="N3">
-        <f>11.71/15.49</f>
-        <v>0.75597159457714658</v>
+      <c r="N3" s="11">
+        <f>B23</f>
+        <v>0.92344863824651802</v>
       </c>
     </row>
     <row r="4" spans="12:15" x14ac:dyDescent="0.35">
       <c r="M4" t="s">
         <v>11</v>
       </c>
-      <c r="N4">
+      <c r="N4" s="9">
         <f>1-N3</f>
-        <v>0.24402840542285342</v>
+        <v>7.6551361753481983E-2</v>
       </c>
     </row>
     <row r="6" spans="12:15" x14ac:dyDescent="0.35">
@@ -703,7 +731,7 @@
       </c>
       <c r="N10" s="5">
         <f>N6/N8*N3</f>
-        <v>0.20699532974404683</v>
+        <v>0.25285282773415407</v>
       </c>
     </row>
     <row r="11" spans="12:15" x14ac:dyDescent="0.35">
@@ -712,7 +740,7 @@
       </c>
       <c r="N11" s="5">
         <f>N6/N8*N4</f>
-        <v>6.6818304562980088E-2</v>
+        <v>2.0960806572872845E-2</v>
       </c>
     </row>
     <row r="12" spans="12:15" x14ac:dyDescent="0.35">
@@ -737,7 +765,7 @@
       </c>
       <c r="N15" s="5">
         <f>N10</f>
-        <v>0.20699532974404683</v>
+        <v>0.25285282773415407</v>
       </c>
     </row>
     <row r="16" spans="12:15" x14ac:dyDescent="0.35">
@@ -749,8 +777,103 @@
       </c>
       <c r="N16" s="5">
         <f>N11</f>
-        <v>6.6818304562980088E-2</v>
-      </c>
+        <v>2.0960806572872845E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="2:39" x14ac:dyDescent="0.35">
+      <c r="B22" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="23" spans="2:39" x14ac:dyDescent="0.35">
+      <c r="B23" s="9">
+        <v>0.92344863824651802</v>
+      </c>
+      <c r="C23" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="24" spans="2:39" x14ac:dyDescent="0.35">
+      <c r="N24" s="6"/>
+      <c r="O24" s="6"/>
+      <c r="P24" s="6"/>
+      <c r="Q24" s="6"/>
+      <c r="R24" s="6"/>
+      <c r="S24" s="6"/>
+      <c r="T24" s="6"/>
+      <c r="U24" s="6"/>
+      <c r="V24" s="6"/>
+      <c r="W24" s="6"/>
+      <c r="X24" s="6"/>
+      <c r="Y24" s="6"/>
+      <c r="Z24" s="6"/>
+      <c r="AA24" s="6"/>
+      <c r="AB24" s="6"/>
+      <c r="AC24" s="6"/>
+      <c r="AD24" s="6"/>
+      <c r="AE24" s="6"/>
+      <c r="AF24" s="6"/>
+      <c r="AG24" s="6"/>
+      <c r="AH24" s="6"/>
+      <c r="AI24" s="6"/>
+      <c r="AJ24" s="6"/>
+      <c r="AK24" s="6"/>
+      <c r="AL24" s="6"/>
+      <c r="AM24" s="6"/>
+    </row>
+    <row r="28" spans="2:39" x14ac:dyDescent="0.35">
+      <c r="N28" s="6"/>
+      <c r="O28" s="6"/>
+      <c r="P28" s="6"/>
+      <c r="Q28" s="6"/>
+      <c r="R28" s="6"/>
+      <c r="S28" s="6"/>
+      <c r="T28" s="6"/>
+      <c r="U28" s="6"/>
+      <c r="V28" s="6"/>
+      <c r="W28" s="6"/>
+      <c r="X28" s="6"/>
+      <c r="Y28" s="6"/>
+      <c r="Z28" s="6"/>
+      <c r="AA28" s="6"/>
+      <c r="AB28" s="6"/>
+      <c r="AC28" s="6"/>
+      <c r="AD28" s="6"/>
+      <c r="AE28" s="6"/>
+      <c r="AF28" s="6"/>
+      <c r="AG28" s="6"/>
+      <c r="AH28" s="6"/>
+      <c r="AI28" s="6"/>
+      <c r="AJ28" s="6"/>
+      <c r="AK28" s="6"/>
+      <c r="AL28" s="6"/>
+      <c r="AM28" s="6"/>
+    </row>
+    <row r="32" spans="2:39" x14ac:dyDescent="0.35">
+      <c r="N32" s="6"/>
+      <c r="O32" s="6"/>
+      <c r="P32" s="6"/>
+      <c r="Q32" s="6"/>
+      <c r="R32" s="6"/>
+      <c r="S32" s="6"/>
+    </row>
+    <row r="34" spans="14:20" x14ac:dyDescent="0.35">
+      <c r="N34" s="9"/>
+      <c r="O34" s="9"/>
+      <c r="P34" s="9"/>
+      <c r="Q34" s="9"/>
+      <c r="R34" s="9"/>
+      <c r="S34" s="9"/>
+      <c r="T34" s="6"/>
+    </row>
+    <row r="35" spans="14:20" x14ac:dyDescent="0.35">
+      <c r="N35" s="9"/>
+      <c r="O35" s="9"/>
+      <c r="P35" s="9"/>
+      <c r="Q35" s="9"/>
+      <c r="R35" s="9"/>
+      <c r="S35" s="9"/>
+      <c r="T35" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1968,103 +2091,103 @@
       </c>
       <c r="G3" s="5">
         <f>1-SUM(G7:G8)</f>
-        <v>0.94523727313859496</v>
+        <v>0.94523727313858963</v>
       </c>
       <c r="H3" s="5">
         <f t="shared" ref="H3:AE3" si="1">1-SUM(H7:H8)</f>
-        <v>0.89047454627718992</v>
+        <v>0.89047454627718103</v>
       </c>
       <c r="I3" s="5">
         <f t="shared" si="1"/>
-        <v>0.83571181941578487</v>
+        <v>0.83571181941578665</v>
       </c>
       <c r="J3" s="5">
         <f t="shared" si="1"/>
-        <v>0.78094909255437983</v>
+        <v>0.78094909255437628</v>
       </c>
       <c r="K3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="L3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="M3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="N3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="O3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="P3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="Q3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="R3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="S3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="T3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="U3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="V3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="W3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="X3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="Y3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="Z3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="AA3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="AB3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="AC3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="AD3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="AE3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
     </row>
     <row r="4" spans="1:31" x14ac:dyDescent="0.35">
@@ -2373,103 +2496,103 @@
       </c>
       <c r="G7" s="5" cm="1">
         <f t="array" ref="G7">TREND(BNEF!$M16:$N16,BNEF!$M$14:$N$14,BHPSbP!G$1)</f>
-        <v>1.3363660912595776E-2</v>
+        <v>4.1921613145756709E-3</v>
       </c>
       <c r="H7" s="5" cm="1">
         <f t="array" ref="H7">TREND(BNEF!$M16:$N16,BNEF!$M$14:$N$14,BHPSbP!H$1)</f>
-        <v>2.6727321825191552E-2</v>
+        <v>8.3843226291495654E-3</v>
       </c>
       <c r="I7" s="5" cm="1">
         <f t="array" ref="I7">TREND(BNEF!$M16:$N16,BNEF!$M$14:$N$14,BHPSbP!I$1)</f>
-        <v>4.0090982737787328E-2</v>
+        <v>1.257648394372346E-2</v>
       </c>
       <c r="J7" s="5" cm="1">
         <f t="array" ref="J7">TREND(BNEF!$M16:$N16,BNEF!$M$14:$N$14,BHPSbP!J$1)</f>
-        <v>5.3454643650383105E-2</v>
+        <v>1.6768645258299131E-2</v>
       </c>
       <c r="K7" s="5" cm="1">
         <f t="array" ref="K7">TREND(BNEF!$M16:$N16,BNEF!$M$14:$N$14,BHPSbP!K$1)</f>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="L7" s="5">
         <f>K7</f>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="M7" s="5">
         <f t="shared" ref="M7:AE7" si="2">L7</f>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="N7" s="5">
         <f t="shared" si="2"/>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="O7" s="5">
         <f t="shared" si="2"/>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="P7" s="5">
         <f t="shared" si="2"/>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="Q7" s="5">
         <f t="shared" si="2"/>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="R7" s="5">
         <f t="shared" si="2"/>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="S7" s="5">
         <f t="shared" si="2"/>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="T7" s="5">
         <f t="shared" si="2"/>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="U7" s="5">
         <f t="shared" si="2"/>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="V7" s="5">
         <f t="shared" si="2"/>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="W7" s="5">
         <f t="shared" si="2"/>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="X7" s="5">
         <f t="shared" si="2"/>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="Y7" s="5">
         <f t="shared" si="2"/>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="Z7" s="5">
         <f t="shared" si="2"/>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="AA7" s="5">
         <f t="shared" si="2"/>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="AB7" s="5">
         <f t="shared" si="2"/>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="AC7" s="5">
         <f t="shared" si="2"/>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="AD7" s="5">
         <f t="shared" si="2"/>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="AE7" s="5">
         <f t="shared" si="2"/>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
     </row>
     <row r="8" spans="1:31" x14ac:dyDescent="0.35">
@@ -2493,103 +2616,103 @@
       </c>
       <c r="G8" s="5" cm="1">
         <f t="array" ref="G8">TREND(BNEF!$M15:$N15,BNEF!$M$14:$N$14,BHPSbP!G$1)</f>
-        <v>4.1399065948809266E-2</v>
+        <v>5.05705655468347E-2</v>
       </c>
       <c r="H8" s="5" cm="1">
         <f t="array" ref="H8">TREND(BNEF!$M15:$N15,BNEF!$M$14:$N$14,BHPSbP!H$1)</f>
-        <v>8.2798131897618532E-2</v>
+        <v>0.1011411310936694</v>
       </c>
       <c r="I8" s="5" cm="1">
         <f t="array" ref="I8">TREND(BNEF!$M15:$N15,BNEF!$M$14:$N$14,BHPSbP!I$1)</f>
-        <v>0.1241971978464278</v>
+        <v>0.15171169664048989</v>
       </c>
       <c r="J8" s="5" cm="1">
         <f t="array" ref="J8">TREND(BNEF!$M15:$N15,BNEF!$M$14:$N$14,BHPSbP!J$1)</f>
-        <v>0.16559626379523706</v>
+        <v>0.20228226218732459</v>
       </c>
       <c r="K8" s="5" cm="1">
         <f t="array" ref="K8">TREND(BNEF!$M15:$N15,BNEF!$M$14:$N$14,BHPSbP!K$1)</f>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="L8" s="5">
         <f>K8</f>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="M8" s="5">
         <f t="shared" ref="M8:AE8" si="3">L8</f>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="N8" s="5">
         <f t="shared" si="3"/>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="O8" s="5">
         <f t="shared" si="3"/>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="P8" s="5">
         <f t="shared" si="3"/>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="Q8" s="5">
         <f t="shared" si="3"/>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="R8" s="5">
         <f t="shared" si="3"/>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="S8" s="5">
         <f t="shared" si="3"/>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="T8" s="5">
         <f t="shared" si="3"/>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="U8" s="5">
         <f t="shared" si="3"/>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="V8" s="5">
         <f t="shared" si="3"/>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="W8" s="5">
         <f t="shared" si="3"/>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="X8" s="5">
         <f t="shared" si="3"/>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="Y8" s="5">
         <f t="shared" si="3"/>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="Z8" s="5">
         <f t="shared" si="3"/>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="AA8" s="5">
         <f t="shared" si="3"/>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="AB8" s="5">
         <f t="shared" si="3"/>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="AC8" s="5">
         <f t="shared" si="3"/>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="AD8" s="5">
         <f t="shared" si="3"/>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="AE8" s="5">
         <f t="shared" si="3"/>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revert "Merge branch 'develop_4.0.5_Jan25Frozen' into develop_4.0.5"
This reverts commit 7520a22cca13a755788ba804722988d6f2c3f7f3, reversing
changes made to 7cd51d1872962a3b3d13dbbe886bf9254c09629a.
</commit_message>
<xml_diff>
--- a/InputData/hydgn/BHPSbP/BAU Hydrogen Production Shr by Pathway.xlsx
+++ b/InputData/hydgn/BHPSbP/BAU Hydrogen Production Shr by Pathway.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\hydgn\BHPSbP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C64BE0A-0A22-4081-AE98-1D3A0E06D094}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0746773-3F94-4C80-9392-DDC2F80141A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1520" yWindow="1520" windowWidth="14400" windowHeight="9340" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="32">
   <si>
     <t>BHPSbP BAU Hydrogen Production Shares by Pathway</t>
   </si>
@@ -157,24 +157,6 @@
   </si>
   <si>
     <t>pgs. 10, 16</t>
-  </si>
-  <si>
-    <t>blue share of clean H2 supply</t>
-  </si>
-  <si>
-    <t>Hydrogen Supply Outlook Update: 10% Cut</t>
-  </si>
-  <si>
-    <t>https://www.bnef.com/insights/38875</t>
-  </si>
-  <si>
-    <t>Blue/green clean hydrogen split</t>
-  </si>
-  <si>
-    <t>Clean hydrogen offtake demand</t>
-  </si>
-  <si>
-    <t>Aggregated expected production from projects; included with permission</t>
   </si>
 </sst>
 </file>
@@ -184,7 +166,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -208,15 +190,8 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -226,12 +201,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.14999847407452621"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -245,12 +214,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -264,14 +232,10 @@
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -297,16 +261,16 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>534092</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>171193</xdr:rowOff>
+      <xdr:colOff>536696</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>70110</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 3">
+        <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{150E1DB1-3649-4488-8F2D-F0C181554476}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D8661492-DC81-408D-BF1C-FD0AB9692D4E}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -322,8 +286,52 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="606136" y="184006"/>
-          <a:ext cx="5989320" cy="3299289"/>
+          <a:off x="609600" y="184150"/>
+          <a:ext cx="6023096" cy="3384810"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>534092</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>171193</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{02F6FC29-38EA-45AA-81F7-E95FC535D07A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="606136" y="3752273"/>
+          <a:ext cx="5989320" cy="3360625"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -598,11 +606,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.7265625" customWidth="1"/>
-    <col min="2" max="2" width="52.6328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
@@ -614,63 +621,28 @@
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="10" t="s">
-        <v>36</v>
+      <c r="B3" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B4" t="s">
-        <v>28</v>
+      <c r="B4" s="3">
+        <v>2025</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B5" s="3">
-        <v>2025</v>
+      <c r="B5" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B6" t="s">
-        <v>29</v>
+      <c r="B6" s="4" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B7" s="4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B8" t="s">
+      <c r="B7" t="s">
         <v>31</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B10" s="10" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B11" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B12" s="3">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B13" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B14" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B15" t="s">
-        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -681,25 +653,25 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3FCF00DD-FBB5-4F2F-A64F-4218B001AAAE}">
-  <dimension ref="B3:AM35"/>
+  <dimension ref="L3:O16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="3" spans="12:15" x14ac:dyDescent="0.35">
       <c r="M3" t="s">
         <v>10</v>
       </c>
-      <c r="N3" s="11">
-        <f>B23</f>
-        <v>0.92344863824651802</v>
+      <c r="N3">
+        <f>11.71/15.49</f>
+        <v>0.75597159457714658</v>
       </c>
     </row>
     <row r="4" spans="12:15" x14ac:dyDescent="0.35">
       <c r="M4" t="s">
         <v>11</v>
       </c>
-      <c r="N4" s="9">
+      <c r="N4">
         <f>1-N3</f>
-        <v>7.6551361753481983E-2</v>
+        <v>0.24402840542285342</v>
       </c>
     </row>
     <row r="6" spans="12:15" x14ac:dyDescent="0.35">
@@ -731,7 +703,7 @@
       </c>
       <c r="N10" s="5">
         <f>N6/N8*N3</f>
-        <v>0.25285282773415407</v>
+        <v>0.20699532974404683</v>
       </c>
     </row>
     <row r="11" spans="12:15" x14ac:dyDescent="0.35">
@@ -740,7 +712,7 @@
       </c>
       <c r="N11" s="5">
         <f>N6/N8*N4</f>
-        <v>2.0960806572872845E-2</v>
+        <v>6.6818304562980088E-2</v>
       </c>
     </row>
     <row r="12" spans="12:15" x14ac:dyDescent="0.35">
@@ -765,7 +737,7 @@
       </c>
       <c r="N15" s="5">
         <f>N10</f>
-        <v>0.25285282773415407</v>
+        <v>0.20699532974404683</v>
       </c>
     </row>
     <row r="16" spans="12:15" x14ac:dyDescent="0.35">
@@ -777,103 +749,8 @@
       </c>
       <c r="N16" s="5">
         <f>N11</f>
-        <v>2.0960806572872845E-2</v>
-      </c>
-    </row>
-    <row r="22" spans="2:39" x14ac:dyDescent="0.35">
-      <c r="B22" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="23" spans="2:39" x14ac:dyDescent="0.35">
-      <c r="B23" s="9">
-        <v>0.92344863824651802</v>
-      </c>
-      <c r="C23" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="24" spans="2:39" x14ac:dyDescent="0.35">
-      <c r="N24" s="6"/>
-      <c r="O24" s="6"/>
-      <c r="P24" s="6"/>
-      <c r="Q24" s="6"/>
-      <c r="R24" s="6"/>
-      <c r="S24" s="6"/>
-      <c r="T24" s="6"/>
-      <c r="U24" s="6"/>
-      <c r="V24" s="6"/>
-      <c r="W24" s="6"/>
-      <c r="X24" s="6"/>
-      <c r="Y24" s="6"/>
-      <c r="Z24" s="6"/>
-      <c r="AA24" s="6"/>
-      <c r="AB24" s="6"/>
-      <c r="AC24" s="6"/>
-      <c r="AD24" s="6"/>
-      <c r="AE24" s="6"/>
-      <c r="AF24" s="6"/>
-      <c r="AG24" s="6"/>
-      <c r="AH24" s="6"/>
-      <c r="AI24" s="6"/>
-      <c r="AJ24" s="6"/>
-      <c r="AK24" s="6"/>
-      <c r="AL24" s="6"/>
-      <c r="AM24" s="6"/>
-    </row>
-    <row r="28" spans="2:39" x14ac:dyDescent="0.35">
-      <c r="N28" s="6"/>
-      <c r="O28" s="6"/>
-      <c r="P28" s="6"/>
-      <c r="Q28" s="6"/>
-      <c r="R28" s="6"/>
-      <c r="S28" s="6"/>
-      <c r="T28" s="6"/>
-      <c r="U28" s="6"/>
-      <c r="V28" s="6"/>
-      <c r="W28" s="6"/>
-      <c r="X28" s="6"/>
-      <c r="Y28" s="6"/>
-      <c r="Z28" s="6"/>
-      <c r="AA28" s="6"/>
-      <c r="AB28" s="6"/>
-      <c r="AC28" s="6"/>
-      <c r="AD28" s="6"/>
-      <c r="AE28" s="6"/>
-      <c r="AF28" s="6"/>
-      <c r="AG28" s="6"/>
-      <c r="AH28" s="6"/>
-      <c r="AI28" s="6"/>
-      <c r="AJ28" s="6"/>
-      <c r="AK28" s="6"/>
-      <c r="AL28" s="6"/>
-      <c r="AM28" s="6"/>
-    </row>
-    <row r="32" spans="2:39" x14ac:dyDescent="0.35">
-      <c r="N32" s="6"/>
-      <c r="O32" s="6"/>
-      <c r="P32" s="6"/>
-      <c r="Q32" s="6"/>
-      <c r="R32" s="6"/>
-      <c r="S32" s="6"/>
-    </row>
-    <row r="34" spans="14:20" x14ac:dyDescent="0.35">
-      <c r="N34" s="9"/>
-      <c r="O34" s="9"/>
-      <c r="P34" s="9"/>
-      <c r="Q34" s="9"/>
-      <c r="R34" s="9"/>
-      <c r="S34" s="9"/>
-      <c r="T34" s="6"/>
-    </row>
-    <row r="35" spans="14:20" x14ac:dyDescent="0.35">
-      <c r="N35" s="9"/>
-      <c r="O35" s="9"/>
-      <c r="P35" s="9"/>
-      <c r="Q35" s="9"/>
-      <c r="R35" s="9"/>
-      <c r="S35" s="9"/>
-      <c r="T35" s="6"/>
+        <v>6.6818304562980088E-2</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2091,103 +1968,103 @@
       </c>
       <c r="G3" s="5">
         <f>1-SUM(G7:G8)</f>
-        <v>0.94523727313858963</v>
+        <v>0.94523727313859496</v>
       </c>
       <c r="H3" s="5">
         <f t="shared" ref="H3:AE3" si="1">1-SUM(H7:H8)</f>
-        <v>0.89047454627718103</v>
+        <v>0.89047454627718992</v>
       </c>
       <c r="I3" s="5">
         <f t="shared" si="1"/>
-        <v>0.83571181941578665</v>
+        <v>0.83571181941578487</v>
       </c>
       <c r="J3" s="5">
         <f t="shared" si="1"/>
-        <v>0.78094909255437628</v>
+        <v>0.78094909255437983</v>
       </c>
       <c r="K3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569296768</v>
+        <v>0.72618636569297479</v>
       </c>
       <c r="L3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569296768</v>
+        <v>0.72618636569297479</v>
       </c>
       <c r="M3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569296768</v>
+        <v>0.72618636569297479</v>
       </c>
       <c r="N3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569296768</v>
+        <v>0.72618636569297479</v>
       </c>
       <c r="O3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569296768</v>
+        <v>0.72618636569297479</v>
       </c>
       <c r="P3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569296768</v>
+        <v>0.72618636569297479</v>
       </c>
       <c r="Q3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569296768</v>
+        <v>0.72618636569297479</v>
       </c>
       <c r="R3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569296768</v>
+        <v>0.72618636569297479</v>
       </c>
       <c r="S3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569296768</v>
+        <v>0.72618636569297479</v>
       </c>
       <c r="T3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569296768</v>
+        <v>0.72618636569297479</v>
       </c>
       <c r="U3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569296768</v>
+        <v>0.72618636569297479</v>
       </c>
       <c r="V3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569296768</v>
+        <v>0.72618636569297479</v>
       </c>
       <c r="W3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569296768</v>
+        <v>0.72618636569297479</v>
       </c>
       <c r="X3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569296768</v>
+        <v>0.72618636569297479</v>
       </c>
       <c r="Y3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569296768</v>
+        <v>0.72618636569297479</v>
       </c>
       <c r="Z3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569296768</v>
+        <v>0.72618636569297479</v>
       </c>
       <c r="AA3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569296768</v>
+        <v>0.72618636569297479</v>
       </c>
       <c r="AB3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569296768</v>
+        <v>0.72618636569297479</v>
       </c>
       <c r="AC3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569296768</v>
+        <v>0.72618636569297479</v>
       </c>
       <c r="AD3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569296768</v>
+        <v>0.72618636569297479</v>
       </c>
       <c r="AE3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569296768</v>
+        <v>0.72618636569297479</v>
       </c>
     </row>
     <row r="4" spans="1:31" x14ac:dyDescent="0.35">
@@ -2496,103 +2373,103 @@
       </c>
       <c r="G7" s="5" cm="1">
         <f t="array" ref="G7">TREND(BNEF!$M16:$N16,BNEF!$M$14:$N$14,BHPSbP!G$1)</f>
-        <v>4.1921613145756709E-3</v>
+        <v>1.3363660912595776E-2</v>
       </c>
       <c r="H7" s="5" cm="1">
         <f t="array" ref="H7">TREND(BNEF!$M16:$N16,BNEF!$M$14:$N$14,BHPSbP!H$1)</f>
-        <v>8.3843226291495654E-3</v>
+        <v>2.6727321825191552E-2</v>
       </c>
       <c r="I7" s="5" cm="1">
         <f t="array" ref="I7">TREND(BNEF!$M16:$N16,BNEF!$M$14:$N$14,BHPSbP!I$1)</f>
-        <v>1.257648394372346E-2</v>
+        <v>4.0090982737787328E-2</v>
       </c>
       <c r="J7" s="5" cm="1">
         <f t="array" ref="J7">TREND(BNEF!$M16:$N16,BNEF!$M$14:$N$14,BHPSbP!J$1)</f>
-        <v>1.6768645258299131E-2</v>
+        <v>5.3454643650383105E-2</v>
       </c>
       <c r="K7" s="5" cm="1">
         <f t="array" ref="K7">TREND(BNEF!$M16:$N16,BNEF!$M$14:$N$14,BHPSbP!K$1)</f>
-        <v>2.0960806572873025E-2</v>
+        <v>6.6818304562978881E-2</v>
       </c>
       <c r="L7" s="5">
         <f>K7</f>
-        <v>2.0960806572873025E-2</v>
+        <v>6.6818304562978881E-2</v>
       </c>
       <c r="M7" s="5">
         <f t="shared" ref="M7:AE7" si="2">L7</f>
-        <v>2.0960806572873025E-2</v>
+        <v>6.6818304562978881E-2</v>
       </c>
       <c r="N7" s="5">
         <f t="shared" si="2"/>
-        <v>2.0960806572873025E-2</v>
+        <v>6.6818304562978881E-2</v>
       </c>
       <c r="O7" s="5">
         <f t="shared" si="2"/>
-        <v>2.0960806572873025E-2</v>
+        <v>6.6818304562978881E-2</v>
       </c>
       <c r="P7" s="5">
         <f t="shared" si="2"/>
-        <v>2.0960806572873025E-2</v>
+        <v>6.6818304562978881E-2</v>
       </c>
       <c r="Q7" s="5">
         <f t="shared" si="2"/>
-        <v>2.0960806572873025E-2</v>
+        <v>6.6818304562978881E-2</v>
       </c>
       <c r="R7" s="5">
         <f t="shared" si="2"/>
-        <v>2.0960806572873025E-2</v>
+        <v>6.6818304562978881E-2</v>
       </c>
       <c r="S7" s="5">
         <f t="shared" si="2"/>
-        <v>2.0960806572873025E-2</v>
+        <v>6.6818304562978881E-2</v>
       </c>
       <c r="T7" s="5">
         <f t="shared" si="2"/>
-        <v>2.0960806572873025E-2</v>
+        <v>6.6818304562978881E-2</v>
       </c>
       <c r="U7" s="5">
         <f t="shared" si="2"/>
-        <v>2.0960806572873025E-2</v>
+        <v>6.6818304562978881E-2</v>
       </c>
       <c r="V7" s="5">
         <f t="shared" si="2"/>
-        <v>2.0960806572873025E-2</v>
+        <v>6.6818304562978881E-2</v>
       </c>
       <c r="W7" s="5">
         <f t="shared" si="2"/>
-        <v>2.0960806572873025E-2</v>
+        <v>6.6818304562978881E-2</v>
       </c>
       <c r="X7" s="5">
         <f t="shared" si="2"/>
-        <v>2.0960806572873025E-2</v>
+        <v>6.6818304562978881E-2</v>
       </c>
       <c r="Y7" s="5">
         <f t="shared" si="2"/>
-        <v>2.0960806572873025E-2</v>
+        <v>6.6818304562978881E-2</v>
       </c>
       <c r="Z7" s="5">
         <f t="shared" si="2"/>
-        <v>2.0960806572873025E-2</v>
+        <v>6.6818304562978881E-2</v>
       </c>
       <c r="AA7" s="5">
         <f t="shared" si="2"/>
-        <v>2.0960806572873025E-2</v>
+        <v>6.6818304562978881E-2</v>
       </c>
       <c r="AB7" s="5">
         <f t="shared" si="2"/>
-        <v>2.0960806572873025E-2</v>
+        <v>6.6818304562978881E-2</v>
       </c>
       <c r="AC7" s="5">
         <f t="shared" si="2"/>
-        <v>2.0960806572873025E-2</v>
+        <v>6.6818304562978881E-2</v>
       </c>
       <c r="AD7" s="5">
         <f t="shared" si="2"/>
-        <v>2.0960806572873025E-2</v>
+        <v>6.6818304562978881E-2</v>
       </c>
       <c r="AE7" s="5">
         <f t="shared" si="2"/>
-        <v>2.0960806572873025E-2</v>
+        <v>6.6818304562978881E-2</v>
       </c>
     </row>
     <row r="8" spans="1:31" x14ac:dyDescent="0.35">
@@ -2616,103 +2493,103 @@
       </c>
       <c r="G8" s="5" cm="1">
         <f t="array" ref="G8">TREND(BNEF!$M15:$N15,BNEF!$M$14:$N$14,BHPSbP!G$1)</f>
-        <v>5.05705655468347E-2</v>
+        <v>4.1399065948809266E-2</v>
       </c>
       <c r="H8" s="5" cm="1">
         <f t="array" ref="H8">TREND(BNEF!$M15:$N15,BNEF!$M$14:$N$14,BHPSbP!H$1)</f>
-        <v>0.1011411310936694</v>
+        <v>8.2798131897618532E-2</v>
       </c>
       <c r="I8" s="5" cm="1">
         <f t="array" ref="I8">TREND(BNEF!$M15:$N15,BNEF!$M$14:$N$14,BHPSbP!I$1)</f>
-        <v>0.15171169664048989</v>
+        <v>0.1241971978464278</v>
       </c>
       <c r="J8" s="5" cm="1">
         <f t="array" ref="J8">TREND(BNEF!$M15:$N15,BNEF!$M$14:$N$14,BHPSbP!J$1)</f>
-        <v>0.20228226218732459</v>
+        <v>0.16559626379523706</v>
       </c>
       <c r="K8" s="5" cm="1">
         <f t="array" ref="K8">TREND(BNEF!$M15:$N15,BNEF!$M$14:$N$14,BHPSbP!K$1)</f>
-        <v>0.25285282773415929</v>
+        <v>0.20699532974404633</v>
       </c>
       <c r="L8" s="5">
         <f>K8</f>
-        <v>0.25285282773415929</v>
+        <v>0.20699532974404633</v>
       </c>
       <c r="M8" s="5">
         <f t="shared" ref="M8:AE8" si="3">L8</f>
-        <v>0.25285282773415929</v>
+        <v>0.20699532974404633</v>
       </c>
       <c r="N8" s="5">
         <f t="shared" si="3"/>
-        <v>0.25285282773415929</v>
+        <v>0.20699532974404633</v>
       </c>
       <c r="O8" s="5">
         <f t="shared" si="3"/>
-        <v>0.25285282773415929</v>
+        <v>0.20699532974404633</v>
       </c>
       <c r="P8" s="5">
         <f t="shared" si="3"/>
-        <v>0.25285282773415929</v>
+        <v>0.20699532974404633</v>
       </c>
       <c r="Q8" s="5">
         <f t="shared" si="3"/>
-        <v>0.25285282773415929</v>
+        <v>0.20699532974404633</v>
       </c>
       <c r="R8" s="5">
         <f t="shared" si="3"/>
-        <v>0.25285282773415929</v>
+        <v>0.20699532974404633</v>
       </c>
       <c r="S8" s="5">
         <f t="shared" si="3"/>
-        <v>0.25285282773415929</v>
+        <v>0.20699532974404633</v>
       </c>
       <c r="T8" s="5">
         <f t="shared" si="3"/>
-        <v>0.25285282773415929</v>
+        <v>0.20699532974404633</v>
       </c>
       <c r="U8" s="5">
         <f t="shared" si="3"/>
-        <v>0.25285282773415929</v>
+        <v>0.20699532974404633</v>
       </c>
       <c r="V8" s="5">
         <f t="shared" si="3"/>
-        <v>0.25285282773415929</v>
+        <v>0.20699532974404633</v>
       </c>
       <c r="W8" s="5">
         <f t="shared" si="3"/>
-        <v>0.25285282773415929</v>
+        <v>0.20699532974404633</v>
       </c>
       <c r="X8" s="5">
         <f t="shared" si="3"/>
-        <v>0.25285282773415929</v>
+        <v>0.20699532974404633</v>
       </c>
       <c r="Y8" s="5">
         <f t="shared" si="3"/>
-        <v>0.25285282773415929</v>
+        <v>0.20699532974404633</v>
       </c>
       <c r="Z8" s="5">
         <f t="shared" si="3"/>
-        <v>0.25285282773415929</v>
+        <v>0.20699532974404633</v>
       </c>
       <c r="AA8" s="5">
         <f t="shared" si="3"/>
-        <v>0.25285282773415929</v>
+        <v>0.20699532974404633</v>
       </c>
       <c r="AB8" s="5">
         <f t="shared" si="3"/>
-        <v>0.25285282773415929</v>
+        <v>0.20699532974404633</v>
       </c>
       <c r="AC8" s="5">
         <f t="shared" si="3"/>
-        <v>0.25285282773415929</v>
+        <v>0.20699532974404633</v>
       </c>
       <c r="AD8" s="5">
         <f t="shared" si="3"/>
-        <v>0.25285282773415929</v>
+        <v>0.20699532974404633</v>
       </c>
       <c r="AE8" s="5">
         <f t="shared" si="3"/>
-        <v>0.25285282773415929</v>
+        <v>0.20699532974404633</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Merge changes from Jan25 frozen branch
</commit_message>
<xml_diff>
--- a/InputData/hydgn/BHPSbP/BAU Hydrogen Production Shr by Pathway.xlsx
+++ b/InputData/hydgn/BHPSbP/BAU Hydrogen Production Shr by Pathway.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\hydgn\BHPSbP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0746773-3F94-4C80-9392-DDC2F80141A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{37FF2600-3BF2-45A0-A141-49EDFBC5DBBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1520" yWindow="1520" windowWidth="14400" windowHeight="9340" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="38">
   <si>
     <t>BHPSbP BAU Hydrogen Production Shares by Pathway</t>
   </si>
@@ -157,6 +157,24 @@
   </si>
   <si>
     <t>pgs. 10, 16</t>
+  </si>
+  <si>
+    <t>blue share of clean H2 supply</t>
+  </si>
+  <si>
+    <t>Hydrogen Supply Outlook Update: 10% Cut</t>
+  </si>
+  <si>
+    <t>https://www.bnef.com/insights/38875</t>
+  </si>
+  <si>
+    <t>Blue/green clean hydrogen split</t>
+  </si>
+  <si>
+    <t>Clean hydrogen offtake demand</t>
+  </si>
+  <si>
+    <t>Aggregated expected production from projects; included with permission</t>
   </si>
 </sst>
 </file>
@@ -166,7 +184,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -190,8 +208,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -201,6 +226,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -214,11 +245,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -232,10 +264,14 @@
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -261,16 +297,16 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>536696</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>70110</xdr:rowOff>
+      <xdr:colOff>534092</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>171193</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2">
+        <xdr:cNvPr id="4" name="Picture 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D8661492-DC81-408D-BF1C-FD0AB9692D4E}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{150E1DB1-3649-4488-8F2D-F0C181554476}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -286,52 +322,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="609600" y="184150"/>
-          <a:ext cx="6023096" cy="3384810"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>534092</xdr:colOff>
-      <xdr:row>37</xdr:row>
-      <xdr:rowOff>171193</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Picture 4">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{02F6FC29-38EA-45AA-81F7-E95FC535D07A}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="606136" y="3752273"/>
-          <a:ext cx="5989320" cy="3360625"/>
+          <a:off x="606136" y="184006"/>
+          <a:ext cx="5989320" cy="3299289"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -606,43 +598,79 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:B15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.7265625" customWidth="1"/>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="2" width="52.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="10" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B4" s="3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B5" s="3">
         <v>2025</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B5" t="s">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B6" s="4" t="s">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B7" s="4" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B7" t="s">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
         <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B10" s="10" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B12" s="3">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -653,28 +681,28 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3FCF00DD-FBB5-4F2F-A64F-4218B001AAAE}">
-  <dimension ref="L3:O16"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="B3:AM35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="3" spans="12:15" x14ac:dyDescent="0.35">
+    <row r="3" spans="12:15" x14ac:dyDescent="0.25">
       <c r="M3" t="s">
         <v>10</v>
       </c>
-      <c r="N3">
-        <f>11.71/15.49</f>
-        <v>0.75597159457714658</v>
-      </c>
-    </row>
-    <row r="4" spans="12:15" x14ac:dyDescent="0.35">
+      <c r="N3" s="11">
+        <f>B23</f>
+        <v>0.92344863824651802</v>
+      </c>
+    </row>
+    <row r="4" spans="12:15" x14ac:dyDescent="0.25">
       <c r="M4" t="s">
         <v>11</v>
       </c>
-      <c r="N4">
+      <c r="N4" s="9">
         <f>1-N3</f>
-        <v>0.24402840542285342</v>
-      </c>
-    </row>
-    <row r="6" spans="12:15" x14ac:dyDescent="0.35">
+        <v>7.6551361753481983E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="12:15" x14ac:dyDescent="0.25">
       <c r="M6" t="s">
         <v>12</v>
       </c>
@@ -685,7 +713,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="12:15" x14ac:dyDescent="0.35">
+    <row r="8" spans="12:15" x14ac:dyDescent="0.25">
       <c r="M8" t="s">
         <v>23</v>
       </c>
@@ -697,30 +725,30 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="12:15" x14ac:dyDescent="0.35">
+    <row r="10" spans="12:15" x14ac:dyDescent="0.25">
       <c r="M10" t="s">
         <v>10</v>
       </c>
       <c r="N10" s="5">
         <f>N6/N8*N3</f>
-        <v>0.20699532974404683</v>
-      </c>
-    </row>
-    <row r="11" spans="12:15" x14ac:dyDescent="0.35">
+        <v>0.25285282773415407</v>
+      </c>
+    </row>
+    <row r="11" spans="12:15" x14ac:dyDescent="0.25">
       <c r="M11" t="s">
         <v>11</v>
       </c>
       <c r="N11" s="5">
         <f>N6/N8*N4</f>
-        <v>6.6818304562980088E-2</v>
-      </c>
-    </row>
-    <row r="12" spans="12:15" x14ac:dyDescent="0.35">
+        <v>2.0960806572872845E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="12:15" x14ac:dyDescent="0.25">
       <c r="M12" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="12:15" x14ac:dyDescent="0.35">
+    <row r="14" spans="12:15" x14ac:dyDescent="0.25">
       <c r="M14">
         <v>2025</v>
       </c>
@@ -728,7 +756,7 @@
         <v>2030</v>
       </c>
     </row>
-    <row r="15" spans="12:15" x14ac:dyDescent="0.35">
+    <row r="15" spans="12:15" x14ac:dyDescent="0.25">
       <c r="L15" t="s">
         <v>26</v>
       </c>
@@ -737,10 +765,10 @@
       </c>
       <c r="N15" s="5">
         <f>N10</f>
-        <v>0.20699532974404683</v>
-      </c>
-    </row>
-    <row r="16" spans="12:15" x14ac:dyDescent="0.35">
+        <v>0.25285282773415407</v>
+      </c>
+    </row>
+    <row r="16" spans="12:15" x14ac:dyDescent="0.25">
       <c r="L16" t="s">
         <v>27</v>
       </c>
@@ -749,8 +777,103 @@
       </c>
       <c r="N16" s="5">
         <f>N11</f>
-        <v>6.6818304562980088E-2</v>
-      </c>
+        <v>2.0960806572872845E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="2:39" x14ac:dyDescent="0.25">
+      <c r="B22" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="23" spans="2:39" x14ac:dyDescent="0.25">
+      <c r="B23" s="9">
+        <v>0.92344863824651802</v>
+      </c>
+      <c r="C23" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="24" spans="2:39" x14ac:dyDescent="0.25">
+      <c r="N24" s="6"/>
+      <c r="O24" s="6"/>
+      <c r="P24" s="6"/>
+      <c r="Q24" s="6"/>
+      <c r="R24" s="6"/>
+      <c r="S24" s="6"/>
+      <c r="T24" s="6"/>
+      <c r="U24" s="6"/>
+      <c r="V24" s="6"/>
+      <c r="W24" s="6"/>
+      <c r="X24" s="6"/>
+      <c r="Y24" s="6"/>
+      <c r="Z24" s="6"/>
+      <c r="AA24" s="6"/>
+      <c r="AB24" s="6"/>
+      <c r="AC24" s="6"/>
+      <c r="AD24" s="6"/>
+      <c r="AE24" s="6"/>
+      <c r="AF24" s="6"/>
+      <c r="AG24" s="6"/>
+      <c r="AH24" s="6"/>
+      <c r="AI24" s="6"/>
+      <c r="AJ24" s="6"/>
+      <c r="AK24" s="6"/>
+      <c r="AL24" s="6"/>
+      <c r="AM24" s="6"/>
+    </row>
+    <row r="28" spans="2:39" x14ac:dyDescent="0.25">
+      <c r="N28" s="6"/>
+      <c r="O28" s="6"/>
+      <c r="P28" s="6"/>
+      <c r="Q28" s="6"/>
+      <c r="R28" s="6"/>
+      <c r="S28" s="6"/>
+      <c r="T28" s="6"/>
+      <c r="U28" s="6"/>
+      <c r="V28" s="6"/>
+      <c r="W28" s="6"/>
+      <c r="X28" s="6"/>
+      <c r="Y28" s="6"/>
+      <c r="Z28" s="6"/>
+      <c r="AA28" s="6"/>
+      <c r="AB28" s="6"/>
+      <c r="AC28" s="6"/>
+      <c r="AD28" s="6"/>
+      <c r="AE28" s="6"/>
+      <c r="AF28" s="6"/>
+      <c r="AG28" s="6"/>
+      <c r="AH28" s="6"/>
+      <c r="AI28" s="6"/>
+      <c r="AJ28" s="6"/>
+      <c r="AK28" s="6"/>
+      <c r="AL28" s="6"/>
+      <c r="AM28" s="6"/>
+    </row>
+    <row r="32" spans="2:39" x14ac:dyDescent="0.25">
+      <c r="N32" s="6"/>
+      <c r="O32" s="6"/>
+      <c r="P32" s="6"/>
+      <c r="Q32" s="6"/>
+      <c r="R32" s="6"/>
+      <c r="S32" s="6"/>
+    </row>
+    <row r="34" spans="14:20" x14ac:dyDescent="0.25">
+      <c r="N34" s="9"/>
+      <c r="O34" s="9"/>
+      <c r="P34" s="9"/>
+      <c r="Q34" s="9"/>
+      <c r="R34" s="9"/>
+      <c r="S34" s="9"/>
+      <c r="T34" s="6"/>
+    </row>
+    <row r="35" spans="14:20" x14ac:dyDescent="0.25">
+      <c r="N35" s="9"/>
+      <c r="O35" s="9"/>
+      <c r="P35" s="9"/>
+      <c r="Q35" s="9"/>
+      <c r="R35" s="9"/>
+      <c r="S35" s="9"/>
+      <c r="T35" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -761,12 +884,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3ED14057-6164-4D1A-BD42-115A681D8E69}">
   <dimension ref="B2:AC13"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="64.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="64.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:29" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>14</v>
       </c>
@@ -852,7 +975,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="3" spans="2:29" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>15</v>
       </c>
@@ -938,7 +1061,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="2:29" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>16</v>
       </c>
@@ -1024,7 +1147,7 @@
         <v>2293830000000</v>
       </c>
     </row>
-    <row r="5" spans="2:29" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>17</v>
       </c>
@@ -1110,7 +1233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="2:29" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>18</v>
       </c>
@@ -1196,7 +1319,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="2:29" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>19</v>
       </c>
@@ -1282,7 +1405,7 @@
         <v>794974000000000</v>
       </c>
     </row>
-    <row r="8" spans="2:29" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>20</v>
       </c>
@@ -1368,7 +1491,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="2:29" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>21</v>
       </c>
@@ -1454,7 +1577,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="2:29" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>22</v>
       </c>
@@ -1540,7 +1663,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="2:29" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>14</v>
       </c>
@@ -1626,7 +1749,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="13" spans="2:29" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>24</v>
       </c>
@@ -1723,12 +1846,12 @@
     <tabColor theme="8" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:AE8"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40.453125" customWidth="1"/>
+    <col min="1" max="1" width="40.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
@@ -1823,7 +1946,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -1947,7 +2070,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1968,106 +2091,106 @@
       </c>
       <c r="G3" s="5">
         <f>1-SUM(G7:G8)</f>
-        <v>0.94523727313859496</v>
+        <v>0.94523727313858963</v>
       </c>
       <c r="H3" s="5">
         <f t="shared" ref="H3:AE3" si="1">1-SUM(H7:H8)</f>
-        <v>0.89047454627718992</v>
+        <v>0.89047454627718103</v>
       </c>
       <c r="I3" s="5">
         <f t="shared" si="1"/>
-        <v>0.83571181941578487</v>
+        <v>0.83571181941578665</v>
       </c>
       <c r="J3" s="5">
         <f t="shared" si="1"/>
-        <v>0.78094909255437983</v>
+        <v>0.78094909255437628</v>
       </c>
       <c r="K3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="L3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="M3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="N3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="O3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="P3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="Q3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="R3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="S3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="T3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="U3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="V3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="W3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="X3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="Y3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="Z3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="AA3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="AB3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="AC3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="AD3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
+        <v>0.72618636569296768</v>
       </c>
       <c r="AE3" s="5">
         <f t="shared" si="1"/>
-        <v>0.72618636569297479</v>
-      </c>
-    </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.35">
+        <v>0.72618636569296768</v>
+      </c>
+    </row>
+    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -2162,7 +2285,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -2257,7 +2380,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2352,7 +2475,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -2373,106 +2496,106 @@
       </c>
       <c r="G7" s="5" cm="1">
         <f t="array" ref="G7">TREND(BNEF!$M16:$N16,BNEF!$M$14:$N$14,BHPSbP!G$1)</f>
-        <v>1.3363660912595776E-2</v>
+        <v>4.1921613145756709E-3</v>
       </c>
       <c r="H7" s="5" cm="1">
         <f t="array" ref="H7">TREND(BNEF!$M16:$N16,BNEF!$M$14:$N$14,BHPSbP!H$1)</f>
-        <v>2.6727321825191552E-2</v>
+        <v>8.3843226291495654E-3</v>
       </c>
       <c r="I7" s="5" cm="1">
         <f t="array" ref="I7">TREND(BNEF!$M16:$N16,BNEF!$M$14:$N$14,BHPSbP!I$1)</f>
-        <v>4.0090982737787328E-2</v>
+        <v>1.257648394372346E-2</v>
       </c>
       <c r="J7" s="5" cm="1">
         <f t="array" ref="J7">TREND(BNEF!$M16:$N16,BNEF!$M$14:$N$14,BHPSbP!J$1)</f>
-        <v>5.3454643650383105E-2</v>
+        <v>1.6768645258299131E-2</v>
       </c>
       <c r="K7" s="5" cm="1">
         <f t="array" ref="K7">TREND(BNEF!$M16:$N16,BNEF!$M$14:$N$14,BHPSbP!K$1)</f>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="L7" s="5">
         <f>K7</f>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="M7" s="5">
         <f t="shared" ref="M7:AE7" si="2">L7</f>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="N7" s="5">
         <f t="shared" si="2"/>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="O7" s="5">
         <f t="shared" si="2"/>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="P7" s="5">
         <f t="shared" si="2"/>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="Q7" s="5">
         <f t="shared" si="2"/>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="R7" s="5">
         <f t="shared" si="2"/>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="S7" s="5">
         <f t="shared" si="2"/>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="T7" s="5">
         <f t="shared" si="2"/>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="U7" s="5">
         <f t="shared" si="2"/>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="V7" s="5">
         <f t="shared" si="2"/>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="W7" s="5">
         <f t="shared" si="2"/>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="X7" s="5">
         <f t="shared" si="2"/>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="Y7" s="5">
         <f t="shared" si="2"/>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="Z7" s="5">
         <f t="shared" si="2"/>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="AA7" s="5">
         <f t="shared" si="2"/>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="AB7" s="5">
         <f t="shared" si="2"/>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="AC7" s="5">
         <f t="shared" si="2"/>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="AD7" s="5">
         <f t="shared" si="2"/>
-        <v>6.6818304562978881E-2</v>
+        <v>2.0960806572873025E-2</v>
       </c>
       <c r="AE7" s="5">
         <f t="shared" si="2"/>
-        <v>6.6818304562978881E-2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.35">
+        <v>2.0960806572873025E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -2493,103 +2616,103 @@
       </c>
       <c r="G8" s="5" cm="1">
         <f t="array" ref="G8">TREND(BNEF!$M15:$N15,BNEF!$M$14:$N$14,BHPSbP!G$1)</f>
-        <v>4.1399065948809266E-2</v>
+        <v>5.05705655468347E-2</v>
       </c>
       <c r="H8" s="5" cm="1">
         <f t="array" ref="H8">TREND(BNEF!$M15:$N15,BNEF!$M$14:$N$14,BHPSbP!H$1)</f>
-        <v>8.2798131897618532E-2</v>
+        <v>0.1011411310936694</v>
       </c>
       <c r="I8" s="5" cm="1">
         <f t="array" ref="I8">TREND(BNEF!$M15:$N15,BNEF!$M$14:$N$14,BHPSbP!I$1)</f>
-        <v>0.1241971978464278</v>
+        <v>0.15171169664048989</v>
       </c>
       <c r="J8" s="5" cm="1">
         <f t="array" ref="J8">TREND(BNEF!$M15:$N15,BNEF!$M$14:$N$14,BHPSbP!J$1)</f>
-        <v>0.16559626379523706</v>
+        <v>0.20228226218732459</v>
       </c>
       <c r="K8" s="5" cm="1">
         <f t="array" ref="K8">TREND(BNEF!$M15:$N15,BNEF!$M$14:$N$14,BHPSbP!K$1)</f>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="L8" s="5">
         <f>K8</f>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="M8" s="5">
         <f t="shared" ref="M8:AE8" si="3">L8</f>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="N8" s="5">
         <f t="shared" si="3"/>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="O8" s="5">
         <f t="shared" si="3"/>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="P8" s="5">
         <f t="shared" si="3"/>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="Q8" s="5">
         <f t="shared" si="3"/>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="R8" s="5">
         <f t="shared" si="3"/>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="S8" s="5">
         <f t="shared" si="3"/>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="T8" s="5">
         <f t="shared" si="3"/>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="U8" s="5">
         <f t="shared" si="3"/>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="V8" s="5">
         <f t="shared" si="3"/>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="W8" s="5">
         <f t="shared" si="3"/>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="X8" s="5">
         <f t="shared" si="3"/>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="Y8" s="5">
         <f t="shared" si="3"/>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="Z8" s="5">
         <f t="shared" si="3"/>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="AA8" s="5">
         <f t="shared" si="3"/>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="AB8" s="5">
         <f t="shared" si="3"/>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="AC8" s="5">
         <f t="shared" si="3"/>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="AD8" s="5">
         <f t="shared" si="3"/>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
       <c r="AE8" s="5">
         <f t="shared" si="3"/>
-        <v>0.20699532974404633</v>
+        <v>0.25285282773415929</v>
       </c>
     </row>
   </sheetData>

</xml_diff>